<commit_message>
fix(cabelos): adiciona Match Masc Capilar e Malbec Cond Anticaspa ao IAF Cabelos
Dois produtos capilares que caiam sem marca e nao contavam como Cabelos:
- 94200 MATCH MASC C H CIEN/CURV (mascara capilar)
- 89784 MALBEC COND TRAT ANTICASPA (condicionador)

Ambos marca oBoticario. Adicionados em produtos (estoqueplanilha.xlsx) e na
lista oficial iaf_cabelos (cabelos_iaf.xlsx). Nao muda % de cabelo atual (os 3
compradores ja contavam por outros produtos), mas corrige classificacao e marca.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/cabelos_iaf.xlsx
+++ b/data/cabelos_iaf.xlsx
@@ -344,7 +344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1036"/>
+  <dimension ref="A1:C1038"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="10.421875" customWidth="1" min="1" max="1"/>
@@ -15894,6 +15894,40 @@
         </is>
       </c>
     </row>
+    <row r="1037">
+      <c r="A1037" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+      <c r="B1037" t="inlineStr">
+        <is>
+          <t>94200</t>
+        </is>
+      </c>
+      <c r="C1037" t="inlineStr">
+        <is>
+          <t>MATCH MASC C H 2AB 3AB CIEN/CURV V2 350g</t>
+        </is>
+      </c>
+    </row>
+    <row r="1038">
+      <c r="A1038" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+      <c r="B1038" t="inlineStr">
+        <is>
+          <t>89784</t>
+        </is>
+      </c>
+      <c r="C1038" t="inlineStr">
+        <is>
+          <t>MALBEC COND TRAT ANTICASPA CUID V4 250ml</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C1028"/>
   <printOptions headings="0" gridLines="0"/>

</xml_diff>

<commit_message>
fix(cabelos): COMBO MATCH conta como cabelo + Siage Cauterizacao combo vira Eudora
- 98399 COMBO MATCH (oBoticario, linha capilar Match) adicionado ao iaf_cabelos:
  nao contava como cabelo (MATCH nao e' palavra-chave do heuristico; nao da' pra
  adicionar 'MATCH' generico por causa do Niina "Perfect Match" que e' make).
  Impacto: +11 clientes cabelo no arquivo (Kauanne +4, Nathalia +1).
- 97446 COMB SIAGE CAUTERIZACAO/FIOS: marca Eudora (estava sem marca; ja contava
  cabelo por ser combo capilar).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/cabelos_iaf.xlsx
+++ b/data/cabelos_iaf.xlsx
@@ -344,7 +344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1038"/>
+  <dimension ref="A1:C1039"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="10.421875" customWidth="1" min="1" max="1"/>
@@ -15928,6 +15928,23 @@
         </is>
       </c>
     </row>
+    <row r="1039">
+      <c r="A1039" t="inlineStr">
+        <is>
+          <t>oBoticário</t>
+        </is>
+      </c>
+      <c r="B1039" t="inlineStr">
+        <is>
+          <t>98399</t>
+        </is>
+      </c>
+      <c r="C1039" t="inlineStr">
+        <is>
+          <t>COMBO MATCH</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C1028"/>
   <printOptions headings="0" gridLines="0"/>

</xml_diff>

<commit_message>
fix(catalogo): cadastra 4 itens sem marca + estojo Siage Pro Cronology no cabelos
- 4 produtos do grupo que caiam sem marca (setor Kauanne):
  86534 EUD MAKE BAT HID -> Eudora; 97462 COMB PULSE -> Eudora;
  96806 COMB VOLPE -> Eudora; 96222 COMB HER CODE -> oBoticario.
- 89383 ESTJ SIAGE PRO CRONOLOGY -> iaf_cabelos (Eudora): estojo de tratamento
  capilar que nao contava (estojos eram excluidos). Edielene passa a contar.

Kauanne final: multimarca 68 (76,4%), make 50 (56,2%), cabelo 50 (56,2%),
zero itens sem marca. 28 testes passam.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/cabelos_iaf.xlsx
+++ b/data/cabelos_iaf.xlsx
@@ -344,7 +344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1039"/>
+  <dimension ref="A1:C1040"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="10.421875" customWidth="1" min="1" max="1"/>
@@ -15945,6 +15945,23 @@
         </is>
       </c>
     </row>
+    <row r="1040">
+      <c r="A1040" t="inlineStr">
+        <is>
+          <t>Eudora</t>
+        </is>
+      </c>
+      <c r="B1040" t="inlineStr">
+        <is>
+          <t>89383</t>
+        </is>
+      </c>
+      <c r="C1040" t="inlineStr">
+        <is>
+          <t>ESTJ SIAGE PRO CRONOLOGY MAES/26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C1028"/>
   <printOptions headings="0" gridLines="0"/>

</xml_diff>